<commit_message>
feat(roguelike): v0.1.2 主线 20-50 局重设计与局级商店规则
落地 Boss 目标倍率、禁牌型/计分 ban、商店槽位与加价等 RunConfig，同步设计文档与通关解锁展示，更新 dist 构建产物。

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/roguelike/现有技能表.xlsx
+++ b/roguelike/现有技能表.xlsx
@@ -1164,17 +1164,8 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -1744,13 +1735,13 @@
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1758,13 +1749,13 @@
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1772,13 +1763,13 @@
       <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="B4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1786,13 +1777,13 @@
       <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="B5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="1" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1800,13 +1791,13 @@
       <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="4" t="s">
+      <c r="B6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="1" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1814,13 +1805,13 @@
       <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="B7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1828,13 +1819,13 @@
       <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="4" t="s">
+      <c r="B8" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1842,13 +1833,13 @@
       <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="4" t="s">
+      <c r="B9" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E9" s="1">
@@ -1859,13 +1850,13 @@
       <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1873,13 +1864,13 @@
       <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="2" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1887,13 +1878,13 @@
       <c r="A12" s="2">
         <v>11</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="2" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1901,13 +1892,13 @@
       <c r="A13" s="2">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="2" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1915,13 +1906,13 @@
       <c r="A14" s="2">
         <v>13</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="2" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1929,13 +1920,13 @@
       <c r="A15" s="1">
         <v>14</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" s="4" t="s">
+      <c r="B15" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="1" t="s">
         <v>33</v>
       </c>
       <c r="E15" s="1">
@@ -1946,13 +1937,13 @@
       <c r="A16" s="1">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C16" s="4" t="s">
+      <c r="B16" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="1" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1960,13 +1951,13 @@
       <c r="A17" s="1">
         <v>16</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C17" s="4" t="s">
+      <c r="B17" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="1" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1974,13 +1965,13 @@
       <c r="A18" s="1">
         <v>17</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="4" t="s">
+      <c r="B18" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="1" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1988,13 +1979,13 @@
       <c r="A19" s="1">
         <v>18</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C19" s="4" t="s">
+      <c r="B19" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="1" t="s">
         <v>41</v>
       </c>
     </row>
@@ -2002,13 +1993,13 @@
       <c r="A20" s="1">
         <v>19</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C20" s="4" t="s">
+      <c r="B20" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="1" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2016,13 +2007,13 @@
       <c r="A21" s="1">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C21" s="4" t="s">
+      <c r="B21" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="1" t="s">
         <v>45</v>
       </c>
     </row>
@@ -2030,13 +2021,13 @@
       <c r="A22" s="1">
         <v>21</v>
       </c>
-      <c r="B22" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C22" s="4" t="s">
+      <c r="B22" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="1" t="s">
         <v>47</v>
       </c>
     </row>
@@ -2044,13 +2035,13 @@
       <c r="A23" s="1">
         <v>22</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C23" s="4" t="s">
+      <c r="B23" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="1" t="s">
         <v>49</v>
       </c>
     </row>
@@ -2058,13 +2049,13 @@
       <c r="A24" s="1">
         <v>23</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C24" s="4" t="s">
+      <c r="B24" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E24" s="1">
@@ -2075,13 +2066,13 @@
       <c r="A25" s="1">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C25" s="4" t="s">
+      <c r="B25" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="1" t="s">
         <v>53</v>
       </c>
       <c r="E25" s="1">
@@ -2092,13 +2083,13 @@
       <c r="A26" s="1">
         <v>25</v>
       </c>
-      <c r="B26" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C26" s="4" t="s">
+      <c r="B26" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="1" t="s">
         <v>55</v>
       </c>
       <c r="E26" s="1">
@@ -2109,13 +2100,13 @@
       <c r="A27" s="1">
         <v>26</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C27" s="4" t="s">
+      <c r="B27" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E27" s="1">
@@ -2126,13 +2117,13 @@
       <c r="A28" s="1">
         <v>27</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C28" s="4" t="s">
+      <c r="B28" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="1" t="s">
         <v>59</v>
       </c>
       <c r="E28" s="1">
@@ -2143,13 +2134,13 @@
       <c r="A29" s="1">
         <v>28</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C29" s="4" t="s">
+      <c r="B29" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="1" t="s">
         <v>61</v>
       </c>
       <c r="E29" s="1">
@@ -2160,13 +2151,13 @@
       <c r="A30" s="1">
         <v>29</v>
       </c>
-      <c r="B30" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C30" s="4" t="s">
+      <c r="B30" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="1" t="s">
         <v>63</v>
       </c>
       <c r="E30" s="1">
@@ -2177,13 +2168,13 @@
       <c r="A31" s="1">
         <v>30</v>
       </c>
-      <c r="B31" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C31" s="4" t="s">
+      <c r="B31" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="1" t="s">
         <v>65</v>
       </c>
       <c r="E31" s="1">
@@ -2194,13 +2185,13 @@
       <c r="A32" s="2">
         <v>31</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="D32" s="2" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2208,13 +2199,13 @@
       <c r="A33" s="2">
         <v>32</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="D33" s="2" t="s">
         <v>69</v>
       </c>
     </row>
@@ -2222,13 +2213,13 @@
       <c r="A34" s="2">
         <v>33</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="2" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2236,13 +2227,13 @@
       <c r="A35" s="2">
         <v>34</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C35" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="D35" s="2" t="s">
         <v>73</v>
       </c>
     </row>
@@ -2250,13 +2241,13 @@
       <c r="A36" s="2">
         <v>35</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="D36" s="2" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2264,13 +2255,13 @@
       <c r="A37" s="2">
         <v>36</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="D37" s="2" t="s">
         <v>77</v>
       </c>
       <c r="E37" s="2">
@@ -2281,13 +2272,13 @@
       <c r="A38" s="2">
         <v>37</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="B38" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C38" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="D38" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -2295,13 +2286,13 @@
       <c r="A39" s="3">
         <v>38</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="D39" s="3" t="s">
         <v>82</v>
       </c>
       <c r="E39" s="3">
@@ -2312,13 +2303,13 @@
       <c r="A40" s="3">
         <v>39</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D40" s="6" t="s">
+      <c r="D40" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E40" s="3">
@@ -2329,13 +2320,13 @@
       <c r="A41" s="2">
         <v>40</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B41" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C41" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="D41" s="2" t="s">
         <v>86</v>
       </c>
       <c r="E41" s="2">
@@ -2346,13 +2337,13 @@
       <c r="A42" s="3">
         <v>41</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D42" s="6" t="s">
+      <c r="D42" s="3" t="s">
         <v>88</v>
       </c>
       <c r="E42" s="3">
@@ -2363,13 +2354,13 @@
       <c r="A43" s="3">
         <v>42</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="D43" s="3" t="s">
         <v>90</v>
       </c>
     </row>
@@ -2377,13 +2368,13 @@
       <c r="A44" s="3">
         <v>43</v>
       </c>
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D44" s="6" t="s">
+      <c r="D44" s="3" t="s">
         <v>92</v>
       </c>
       <c r="E44" s="3">
@@ -2394,13 +2385,13 @@
       <c r="A45" s="3">
         <v>44</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="D45" s="3" t="s">
         <v>94</v>
       </c>
       <c r="E45" s="3">
@@ -2411,13 +2402,13 @@
       <c r="A46" s="2">
         <v>45</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="C46" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D46" s="5" t="s">
+      <c r="D46" s="2" t="s">
         <v>96</v>
       </c>
       <c r="E46" s="2">
@@ -2428,13 +2419,13 @@
       <c r="A47" s="2">
         <v>46</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="B47" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="C47" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="D47" s="5" t="s">
+      <c r="D47" s="2" t="s">
         <v>98</v>
       </c>
       <c r="E47" s="2">
@@ -2445,13 +2436,13 @@
       <c r="A48" s="3">
         <v>47</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C48" s="6" t="s">
+      <c r="C48" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="D48" s="6" t="s">
+      <c r="D48" s="3" t="s">
         <v>100</v>
       </c>
       <c r="E48" s="3">
@@ -2462,13 +2453,13 @@
       <c r="A49" s="3">
         <v>48</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="C49" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D49" s="6" t="s">
+      <c r="D49" s="3" t="s">
         <v>102</v>
       </c>
       <c r="E49" s="3">
@@ -2479,13 +2470,13 @@
       <c r="A50" s="3">
         <v>49</v>
       </c>
-      <c r="B50" s="6" t="s">
+      <c r="B50" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C50" s="6" t="s">
+      <c r="C50" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="D50" s="6" t="s">
+      <c r="D50" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E50" s="3">
@@ -2496,13 +2487,13 @@
       <c r="A51" s="3">
         <v>50</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C51" s="6" t="s">
+      <c r="C51" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="D51" s="6" t="s">
+      <c r="D51" s="3" t="s">
         <v>106</v>
       </c>
       <c r="E51" s="3">
@@ -2513,13 +2504,13 @@
       <c r="A52" s="3">
         <v>51</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B52" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C52" s="6" t="s">
+      <c r="C52" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="D52" s="6" t="s">
+      <c r="D52" s="3" t="s">
         <v>108</v>
       </c>
       <c r="E52" s="3">
@@ -2530,13 +2521,13 @@
       <c r="A53" s="3">
         <v>52</v>
       </c>
-      <c r="B53" s="6" t="s">
+      <c r="B53" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C53" s="6" t="s">
+      <c r="C53" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="D53" s="6" t="s">
+      <c r="D53" s="3" t="s">
         <v>110</v>
       </c>
       <c r="E53" s="3">
@@ -2547,13 +2538,13 @@
       <c r="A54" s="3">
         <v>53</v>
       </c>
-      <c r="B54" s="6" t="s">
+      <c r="B54" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C54" s="6" t="s">
+      <c r="C54" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="D54" s="6" t="s">
+      <c r="D54" s="3" t="s">
         <v>112</v>
       </c>
     </row>
@@ -2561,13 +2552,13 @@
       <c r="A55" s="3">
         <v>54</v>
       </c>
-      <c r="B55" s="6" t="s">
+      <c r="B55" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C55" s="6" t="s">
+      <c r="C55" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D55" s="6" t="s">
+      <c r="D55" s="3" t="s">
         <v>114</v>
       </c>
     </row>
@@ -2575,13 +2566,13 @@
       <c r="A56" s="3">
         <v>55</v>
       </c>
-      <c r="B56" s="6" t="s">
+      <c r="B56" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C56" s="6" t="s">
+      <c r="C56" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D56" s="6" t="s">
+      <c r="D56" s="3" t="s">
         <v>116</v>
       </c>
     </row>
@@ -2589,13 +2580,13 @@
       <c r="A57" s="3">
         <v>56</v>
       </c>
-      <c r="B57" s="6" t="s">
+      <c r="B57" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C57" s="6" t="s">
+      <c r="C57" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D57" s="6" t="s">
+      <c r="D57" s="3" t="s">
         <v>118</v>
       </c>
       <c r="E57" s="3">
@@ -2606,13 +2597,13 @@
       <c r="A58" s="3">
         <v>57</v>
       </c>
-      <c r="B58" s="6" t="s">
+      <c r="B58" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C58" s="6" t="s">
+      <c r="C58" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="D58" s="6" t="s">
+      <c r="D58" s="3" t="s">
         <v>120</v>
       </c>
     </row>
@@ -2620,13 +2611,13 @@
       <c r="A59" s="3">
         <v>58</v>
       </c>
-      <c r="B59" s="6" t="s">
+      <c r="B59" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C59" s="6" t="s">
+      <c r="C59" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="D59" s="6" t="s">
+      <c r="D59" s="3" t="s">
         <v>122</v>
       </c>
     </row>
@@ -2634,13 +2625,13 @@
       <c r="A60" s="3">
         <v>59</v>
       </c>
-      <c r="B60" s="6" t="s">
+      <c r="B60" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C60" s="6" t="s">
+      <c r="C60" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="D60" s="6" t="s">
+      <c r="D60" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E60" s="3">
@@ -2651,13 +2642,13 @@
       <c r="A61" s="3">
         <v>60</v>
       </c>
-      <c r="B61" s="6" t="s">
+      <c r="B61" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C61" s="6" t="s">
+      <c r="C61" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="D61" s="6" t="s">
+      <c r="D61" s="3" t="s">
         <v>126</v>
       </c>
       <c r="E61" s="3">
@@ -2668,13 +2659,13 @@
       <c r="A62" s="2">
         <v>61</v>
       </c>
-      <c r="B62" s="5" t="s">
+      <c r="B62" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C62" s="5" t="s">
+      <c r="C62" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D62" s="5" t="s">
+      <c r="D62" s="2" t="s">
         <v>128</v>
       </c>
     </row>
@@ -2682,13 +2673,13 @@
       <c r="A63" s="1">
         <v>62</v>
       </c>
-      <c r="B63" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C63" s="4" t="s">
+      <c r="B63" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D63" s="4" t="s">
+      <c r="D63" s="1" t="s">
         <v>130</v>
       </c>
       <c r="E63" s="1">
@@ -2699,13 +2690,13 @@
       <c r="A64" s="1">
         <v>63</v>
       </c>
-      <c r="B64" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C64" s="4" t="s">
+      <c r="B64" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="D64" s="4" t="s">
+      <c r="D64" s="1" t="s">
         <v>132</v>
       </c>
       <c r="E64" s="1">
@@ -2716,13 +2707,13 @@
       <c r="A65" s="2">
         <v>64</v>
       </c>
-      <c r="B65" s="5" t="s">
+      <c r="B65" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C65" s="5" t="s">
+      <c r="C65" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="D65" s="5" t="s">
+      <c r="D65" s="2" t="s">
         <v>134</v>
       </c>
       <c r="E65" s="2">
@@ -2733,13 +2724,13 @@
       <c r="A66" s="2">
         <v>65</v>
       </c>
-      <c r="B66" s="5" t="s">
+      <c r="B66" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C66" s="5" t="s">
+      <c r="C66" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="D66" s="5" t="s">
+      <c r="D66" s="2" t="s">
         <v>136</v>
       </c>
       <c r="E66" s="2">
@@ -2750,13 +2741,13 @@
       <c r="A67" s="2">
         <v>66</v>
       </c>
-      <c r="B67" s="5" t="s">
+      <c r="B67" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C67" s="5" t="s">
+      <c r="C67" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="D67" s="5" t="s">
+      <c r="D67" s="2" t="s">
         <v>138</v>
       </c>
       <c r="E67" s="2">
@@ -2767,13 +2758,13 @@
       <c r="A68" s="2">
         <v>67</v>
       </c>
-      <c r="B68" s="5" t="s">
+      <c r="B68" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C68" s="5" t="s">
+      <c r="C68" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D68" s="5" t="s">
+      <c r="D68" s="2" t="s">
         <v>140</v>
       </c>
       <c r="E68" s="2">
@@ -2784,13 +2775,13 @@
       <c r="A69" s="2">
         <v>68</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="B69" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C69" s="5" t="s">
+      <c r="C69" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="D69" s="5" t="s">
+      <c r="D69" s="2" t="s">
         <v>142</v>
       </c>
       <c r="E69" s="2">
@@ -2801,13 +2792,13 @@
       <c r="A70" s="2">
         <v>69</v>
       </c>
-      <c r="B70" s="5" t="s">
+      <c r="B70" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C70" s="5" t="s">
+      <c r="C70" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D70" s="5" t="s">
+      <c r="D70" s="2" t="s">
         <v>144</v>
       </c>
       <c r="E70" s="2">
@@ -2818,13 +2809,13 @@
       <c r="A71" s="1">
         <v>70</v>
       </c>
-      <c r="B71" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C71" s="4" t="s">
+      <c r="B71" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C71" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="D71" s="4" t="s">
+      <c r="D71" s="1" t="s">
         <v>146</v>
       </c>
     </row>
@@ -2832,13 +2823,13 @@
       <c r="A72" s="1">
         <v>71</v>
       </c>
-      <c r="B72" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C72" s="4" t="s">
+      <c r="B72" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C72" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D72" s="4" t="s">
+      <c r="D72" s="1" t="s">
         <v>148</v>
       </c>
     </row>
@@ -2846,13 +2837,13 @@
       <c r="A73" s="1">
         <v>72</v>
       </c>
-      <c r="B73" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C73" s="4" t="s">
+      <c r="B73" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C73" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="D73" s="4" t="s">
+      <c r="D73" s="1" t="s">
         <v>150</v>
       </c>
       <c r="E73" s="1">
@@ -2863,13 +2854,13 @@
       <c r="A74" s="1">
         <v>73</v>
       </c>
-      <c r="B74" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C74" s="4" t="s">
+      <c r="B74" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C74" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="D74" s="4" t="s">
+      <c r="D74" s="1" t="s">
         <v>152</v>
       </c>
       <c r="E74" s="1">
@@ -2880,13 +2871,13 @@
       <c r="A75" s="3">
         <v>74</v>
       </c>
-      <c r="B75" s="6" t="s">
+      <c r="B75" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C75" s="6" t="s">
+      <c r="C75" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="D75" s="6" t="s">
+      <c r="D75" s="3" t="s">
         <v>154</v>
       </c>
       <c r="E75" s="3">
@@ -2897,13 +2888,13 @@
       <c r="A76" s="1">
         <v>75</v>
       </c>
-      <c r="B76" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C76" s="4" t="s">
+      <c r="B76" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C76" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="D76" s="4" t="s">
+      <c r="D76" s="1" t="s">
         <v>156</v>
       </c>
     </row>
@@ -2911,13 +2902,13 @@
       <c r="A77" s="2">
         <v>76</v>
       </c>
-      <c r="B77" s="5" t="s">
+      <c r="B77" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C77" s="5" t="s">
+      <c r="C77" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="D77" s="5" t="s">
+      <c r="D77" s="2" t="s">
         <v>158</v>
       </c>
       <c r="E77" s="2">
@@ -2928,13 +2919,13 @@
       <c r="A78" s="1">
         <v>77</v>
       </c>
-      <c r="B78" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C78" s="4" t="s">
+      <c r="B78" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C78" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D78" s="4" t="s">
+      <c r="D78" s="1" t="s">
         <v>160</v>
       </c>
       <c r="E78" s="1">
@@ -2945,13 +2936,13 @@
       <c r="A79" s="2">
         <v>78</v>
       </c>
-      <c r="B79" s="5" t="s">
+      <c r="B79" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C79" s="5" t="s">
+      <c r="C79" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="D79" s="5" t="s">
+      <c r="D79" s="2" t="s">
         <v>162</v>
       </c>
       <c r="E79" s="2">
@@ -2962,13 +2953,13 @@
       <c r="A80" s="2">
         <v>79</v>
       </c>
-      <c r="B80" s="5" t="s">
+      <c r="B80" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C80" s="5" t="s">
+      <c r="C80" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="D80" s="5" t="s">
+      <c r="D80" s="2" t="s">
         <v>164</v>
       </c>
       <c r="E80" s="2">
@@ -2979,13 +2970,13 @@
       <c r="A81" s="2">
         <v>80</v>
       </c>
-      <c r="B81" s="5" t="s">
+      <c r="B81" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C81" s="5" t="s">
+      <c r="C81" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="D81" s="5" t="s">
+      <c r="D81" s="2" t="s">
         <v>166</v>
       </c>
       <c r="E81" s="2">

</xml_diff>